<commit_message>
Victor app-report fixes: Home-tab back-link, composite PMID render, drop NCCD_2018 from NOT_IN_NCCD primary refs, VCD citation clarification, ## markdown render
</commit_message>
<xml_diff>
--- a/data/RCDome_Decoder_53.xlsx
+++ b/data/RCDome_Decoder_53.xlsx
@@ -1388,7 +1388,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>17562483;29362479</t>
+          <t>17562483</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>36864290;29362479</t>
+          <t>36864290</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>24726643;29362479</t>
+          <t>24726643</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>23483560;29362479</t>
+          <t>23483560</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>33705288;29362479</t>
+          <t>33705288</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -7272,7 +7272,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>31827074;29362479</t>
+          <t>31827074</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>29255269;29362479</t>
+          <t>29255269</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -8364,7 +8364,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>11121041;29362479</t>
+          <t>11121041</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Kosta et al. 2004</t>
+          <t>Kosta et al. 2004 — name source; describes a non-vacuolar pathway</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">

</xml_diff>

<commit_message>
Victor fixes A+B: clarify composite NCCD citation + VCD plant/Dictyostelium citation
</commit_message>
<xml_diff>
--- a/data/RCDome_Decoder_53.xlsx
+++ b/data/RCDome_Decoder_53.xlsx
@@ -9633,7 +9633,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Composite of Cellular senescence (PMID 29362479) + Autophagy (PMID 36864290)</t>
+          <t>Composite of Cellular senescence (NCCD_2018; PMID 29362479) + Autophagy (PMID 36864290) — composite pathway label, not a distinct NCCD entity</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Kosta et al. 2004 — name source; describes a non-vacuolar pathway</t>
+          <t>Kosta et al. 2004 (Dictyostelium — name source; non-vacuolar pathway); plant context: Minina 2013 (PMID 24344187), Feng 2022 (PMID 35390283)</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">

</xml_diff>

<commit_message>
§9 Lysoptosis L5->L2 (SUBTYPE) + matrix decoder-column re-sync (fix 10 OP drift + 19 category case) + landing page counts
</commit_message>
<xml_diff>
--- a/data/RCDome_Decoder_53.xlsx
+++ b/data/RCDome_Decoder_53.xlsx
@@ -4841,7 +4841,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>LEGACY</t>
+          <t>SUBTYPE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>A lysosome-dependent cell-death process (legacy term) demarcated by lysosomal membrane permeabilization and cathepsin-dependent cytoplasmic proteolysis, executed when serpin inhibition is absent.</t>
+          <t>A lysosome-dependent cell-death subtype demarcated by serpin/SERPINB3-moderated lysosomal membrane permeabilization and cathepsin-L-dependent cytoplasmic proteolysis, executed in the absence of neutralizing endogenous serpin inhibition.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>legacy</t>
+          <t>supported</t>
         </is>
       </c>
       <c r="AI25" t="inlineStr">

</xml_diff>

<commit_message>
Victor V027 protocol: full triage + fixes (46 done, 3 deferred); figures 1/2/3/S1/S3 regenerated + legends aligned; matrix/decoder/MSigDB synced; README/CHANGELOG updated
</commit_message>
<xml_diff>
--- a/data/RCDome_Decoder_53.xlsx
+++ b/data/RCDome_Decoder_53.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -663,6 +664,7 @@
           <t>29248440;36640329</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>pH-dependent death under alkaline conditions; NF-kB/CA9-dependent</t>
@@ -728,6 +730,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -778,9 +781,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
@@ -820,6 +824,7 @@
           <t>A contextual cell-death process triggered by ammonia, demarcated by cytoplasmic vacuolation, and detoxified via arginase-mediated urea production with L-glutamine protection.</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -840,6 +845,8 @@
           <t>12388179</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
           <t>arginase; L-glutamine</t>
@@ -900,6 +907,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -957,7 +965,7 @@
       </c>
       <c r="AK3" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL3" t="inlineStr">
@@ -1154,7 +1162,7 @@
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
@@ -1194,6 +1202,7 @@
           <t>A syncretic cell death variant sharing features of apoptosis and necrosis, triggered by high-dose mitochondrial insult and demarcated by incomplete execution of the apoptotic program, with intracellular ATP as a determinant.</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -1214,6 +1223,8 @@
           <t>10567915</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>caspase-3; respiratory chain complex III</t>
@@ -1274,6 +1285,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -1331,7 +1343,7 @@
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
@@ -1466,6 +1478,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -1516,9 +1529,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ6" t="inlineStr"/>
       <c r="AK6" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL6" t="inlineStr">
@@ -1583,6 +1597,8 @@
           <t>15451440</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr">
         <is>
           <t>CD95/Fas, FADD, caspase-8</t>
@@ -1675,7 +1691,7 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
@@ -1705,7 +1721,7 @@
       </c>
       <c r="AK7" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL7" t="inlineStr">
@@ -1770,6 +1786,8 @@
           <t>12186923</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr">
         <is>
           <t>Bcl-2, Bcl-xL, Bax</t>
@@ -1862,7 +1880,7 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1892,7 +1910,7 @@
       </c>
       <c r="AK8" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL8" t="inlineStr">
@@ -2027,6 +2045,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -2077,9 +2096,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL9" t="inlineStr">
@@ -2144,6 +2164,8 @@
           <t>30568239</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
           <t>autophagy machinery</t>
@@ -2236,7 +2258,7 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -2259,9 +2281,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ10" t="inlineStr"/>
       <c r="AK10" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL10" t="inlineStr">
@@ -2458,7 +2481,7 @@
       </c>
       <c r="AK11" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL11" t="inlineStr">
@@ -2523,6 +2546,7 @@
           <t>23140366;29362479</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>Stable cell cycle arrest with metabolic activity; SASP secretion</t>
@@ -2643,9 +2667,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL12" t="inlineStr">
@@ -2685,6 +2710,7 @@
           <t>A terminal differentiation program of keratinocytes producing the cornified (keratinized) barrier and culminating in a specialized form of programmed cell death.</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -2710,6 +2736,7 @@
           <t>15803139</t>
         </is>
       </c>
+      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
           <t>keratins, transglutaminases, lipids</t>
@@ -2770,6 +2797,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -2820,9 +2848,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL13" t="inlineStr">
@@ -2957,6 +2986,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -3007,9 +3037,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ14" t="inlineStr"/>
       <c r="AK14" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL14" t="inlineStr">
@@ -3144,6 +3175,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -3194,9 +3226,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ15" t="inlineStr"/>
       <c r="AK15" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL15" t="inlineStr">
@@ -3393,7 +3426,7 @@
       </c>
       <c r="AK16" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL16" t="inlineStr">
@@ -3550,7 +3583,7 @@
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Entotic cell death (death) originating from entosis (cell-in-cell process); entosis is the source/process term.</t>
+          <t>Use entotic cell death as the canonical concept name. [2]</t>
         </is>
       </c>
       <c r="AD17" t="inlineStr">
@@ -3583,9 +3616,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ17" t="inlineStr"/>
       <c r="AK17" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL17" t="inlineStr">
@@ -3650,6 +3684,7 @@
           <t>35468130</t>
         </is>
       </c>
+      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>Novel cell death reported in gut enterocyte turnover</t>
@@ -3715,6 +3750,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -3765,9 +3801,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL18" t="inlineStr">
@@ -3807,6 +3844,7 @@
           <t>A cell-type-specific form of regulated cell death of erythrocytes, demarcated by cell shrinkage, membrane blebbing, calpain activation and phosphatidylserine exposure, and triggered by oxidative stress via prostaglandin E2/Ca2+ and phospholipase A2/ceramide pathways.</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -3827,6 +3865,8 @@
           <t>16910766</t>
         </is>
       </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr">
         <is>
           <t>Ca2+ channels, ceramide, calpain, erythropoietin</t>
@@ -3887,6 +3927,7 @@
           <t>DRAFT_CANDIDATE</t>
         </is>
       </c>
+      <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -3937,9 +3978,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ19" t="inlineStr"/>
       <c r="AK19" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL19" t="inlineStr">
@@ -4004,6 +4046,7 @@
           <t>22632970;28985560</t>
         </is>
       </c>
+      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>Iron-dependent lipid peroxide accumulation</t>
@@ -4124,9 +4167,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ20" t="inlineStr"/>
       <c r="AK20" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL20" t="inlineStr">
@@ -4166,6 +4210,7 @@
           <t>A form of regulated cell death demarcated by cytoplasmic vacuolization with fused-lysosome-associated termination, triggered by Bergeyella cardium infection and inhibited by sodium-channel blockade.</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -4186,6 +4231,8 @@
           <t>41115953</t>
         </is>
       </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr">
         <is>
           <t>SLC9A9; sodium channels</t>
@@ -4246,6 +4293,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -4296,9 +4344,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ21" t="inlineStr"/>
       <c r="AK21" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL21" t="inlineStr">
@@ -4338,6 +4387,7 @@
           <t>A taxon-specific programmed cell death of plant cells at infection sites, restricting pathogen spread.</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>PRE_PUBMED</t>
@@ -4358,6 +4408,9 @@
           <t>31305008</t>
         </is>
       </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>No</t>
@@ -4413,6 +4466,7 @@
           <t>PRE_PUBMED</t>
         </is>
       </c>
+      <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -4463,9 +4517,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ22" t="inlineStr"/>
       <c r="AK22" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL22" t="inlineStr">
@@ -4530,6 +4585,7 @@
           <t>23157435;27748397</t>
         </is>
       </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>Dying cells expose/release DAMPs activating adaptive immunity</t>
@@ -4650,9 +4706,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ23" t="inlineStr"/>
       <c r="AK23" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL23" t="inlineStr">
@@ -4692,6 +4749,7 @@
           <t>A taxon-specific, caspase-independent (ced-3-independent) non-apoptotic developmental cell death of the Caenorhabditis elegans linker cell, demarcated by nuclear crenellation and organelle swelling, and controlled by let-7 and LIN-29.</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -4712,6 +4770,8 @@
           <t>17199042</t>
         </is>
       </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr">
         <is>
           <t>let-7; LIN-29</t>
@@ -4772,6 +4832,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -4822,9 +4883,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ24" t="inlineStr"/>
       <c r="AK24" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL24" t="inlineStr">
@@ -4864,6 +4926,7 @@
           <t>A lysosome-dependent cell-death subtype demarcated by serpin/SERPINB3-moderated lysosomal membrane permeabilization and cathepsin-L-dependent cytoplasmic proteolysis, executed in the absence of neutralizing endogenous serpin inhibition.</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -4884,6 +4947,8 @@
           <t>35022507</t>
         </is>
       </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr">
         <is>
           <t>cathepsins (L); SERPINB3</t>
@@ -4944,6 +5009,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -5001,7 +5067,7 @@
       </c>
       <c r="AK25" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL25" t="inlineStr">
@@ -5066,6 +5132,8 @@
           <t>30125440</t>
         </is>
       </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr">
         <is>
           <t>cathepsin B, L</t>
@@ -5158,7 +5226,7 @@
       </c>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF26" t="inlineStr">
@@ -5188,7 +5256,7 @@
       </c>
       <c r="AK26" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL26" t="inlineStr">
@@ -5378,9 +5446,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ27" t="inlineStr"/>
       <c r="AK27" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL27" t="inlineStr">
@@ -5420,6 +5489,7 @@
           <t>A regulated non-apoptotic, lysosomal zinc-dependent cell-death process (emerging concept).</t>
         </is>
       </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -5445,6 +5515,7 @@
           <t>37550363</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr">
         <is>
           <t>lysosomal zinc</t>
@@ -5505,6 +5576,7 @@
           <t>DRAFT_CANDIDATE</t>
         </is>
       </c>
+      <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -5562,7 +5634,7 @@
       </c>
       <c r="AK28" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL28" t="inlineStr">
@@ -5602,6 +5674,7 @@
           <t>An umbrella term for metal-ion-based regulated cell death, encompassing ferroptosis, cuproptosis, lysozincrosis, manganism, calcicoptosis and necrosis by sodium overload.</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -5622,6 +5695,8 @@
           <t>41094656</t>
         </is>
       </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr">
         <is>
           <t>metal ions (Fe, Cu, Zn, Mn, Ca, Na)</t>
@@ -5682,6 +5757,7 @@
           <t>DRAFT_CANDIDATE</t>
         </is>
       </c>
+      <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -5739,7 +5815,7 @@
       </c>
       <c r="AK29" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL29" t="inlineStr">
@@ -5804,6 +5880,7 @@
           <t>24726643</t>
         </is>
       </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>Non-apoptotic death with macropinosome-derived vacuoles; Ras/Rac1-driven</t>
@@ -5869,6 +5946,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -5919,9 +5997,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ30" t="inlineStr"/>
       <c r="AK30" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL30" t="inlineStr">
@@ -6056,6 +6135,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -6106,9 +6186,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ31" t="inlineStr"/>
       <c r="AK31" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL31" t="inlineStr">
@@ -6173,6 +6254,7 @@
           <t>33705288</t>
         </is>
       </c>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>Selective elimination of damaged mitochondria (organelle-level quality control)</t>
@@ -6238,6 +6320,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -6288,9 +6371,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ32" t="inlineStr"/>
       <c r="AK32" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL32" t="inlineStr">
@@ -6355,6 +6439,7 @@
           <t>15077146;29362479</t>
         </is>
       </c>
+      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>Oncosuppressive sensor of aberrant mitosis and genomic instability</t>
@@ -6475,9 +6560,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ33" t="inlineStr"/>
       <c r="AK33" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL33" t="inlineStr">
@@ -6542,6 +6628,9 @@
           <t>6027879</t>
         </is>
       </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>not specified</t>
@@ -6629,7 +6718,7 @@
       </c>
       <c r="AE34" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF34" t="inlineStr">
@@ -6659,7 +6748,7 @@
       </c>
       <c r="AK34" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL34" t="inlineStr">
@@ -6699,6 +6788,7 @@
           <t>A lytic cell-death modality triggered by the synergism of innate-immune and metabolic signals, demarcated by BAX/BAK1/BID-dependent mitochondrial oxidative stress at the plasma membrane and culminating in membrane lysis.</t>
         </is>
       </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -6719,6 +6809,8 @@
           <t>41317732</t>
         </is>
       </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr">
         <is>
           <t>BAX, BAK1, BID, mTORC2</t>
@@ -6779,6 +6871,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -6796,7 +6889,7 @@
       </c>
       <c r="AC35" t="inlineStr">
         <is>
-          <t>Candidate modality (G1+G2 passed; G2 by CRISPR/Cas9 Bax/Bak1/Bid triple-KO resistance, PMC12875127; distinct from MPT (CsA/CypD) and NLRP3); G5 replication pending; human.</t>
+          <t>Candidate modality (BG1+BG2 passed; BG2 by CRISPR/Cas9 Bax/Bak1/Bid triple-KO resistance, PMC12875127; distinct from MPT (CsA/CypD) and NLRP3); BG5 replication pending; human.</t>
         </is>
       </c>
       <c r="AD35" t="inlineStr">
@@ -6829,9 +6922,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ35" t="inlineStr"/>
       <c r="AK35" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL35" t="inlineStr">
@@ -6896,6 +6990,8 @@
           <t>27161573</t>
         </is>
       </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr">
         <is>
           <t>permeability transition pore complex (PTPC)</t>
@@ -6988,7 +7084,7 @@
       </c>
       <c r="AE36" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF36" t="inlineStr">
@@ -7018,7 +7114,7 @@
       </c>
       <c r="AK36" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL36" t="inlineStr">
@@ -7215,7 +7311,7 @@
       </c>
       <c r="AK37" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL37" t="inlineStr">
@@ -7350,6 +7446,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y38" t="inlineStr"/>
       <c r="Z38" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -7407,7 +7504,7 @@
       </c>
       <c r="AK38" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL38" t="inlineStr">
@@ -7447,6 +7544,7 @@
           <t>A necrotic cell-death modality caused by sodium overload, executed via persistent activation of the TRPM4 cation channel by necrocide 1 (NC1).</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -7467,6 +7565,8 @@
           <t>39915626</t>
         </is>
       </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr">
         <is>
           <t>TRPM4, Na+, NC1</t>
@@ -7527,6 +7627,7 @@
           <t>DRAFT_CANDIDATE</t>
         </is>
       </c>
+      <c r="Y39" t="inlineStr"/>
       <c r="Z39" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -7544,7 +7645,7 @@
       </c>
       <c r="AC39" t="inlineStr">
         <is>
-          <t>Candidate modality (G1+G2 passed); G5 replication pending; human TRPM4-specific.</t>
+          <t>Candidate modality (BG1+BG2 passed); BG5 replication pending; human TRPM4-specific.</t>
         </is>
       </c>
       <c r="AD39" t="inlineStr">
@@ -7577,9 +7678,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ39" t="inlineStr"/>
       <c r="AK39" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL39" t="inlineStr">
@@ -7736,7 +7838,7 @@
       </c>
       <c r="AC40" t="inlineStr">
         <is>
-          <t>NETotic cell death (death) associated with NETosis (NET-release process); NETosis is the source/process term.</t>
+          <t>Retain as a distinct regulated-necrosis modality. [2, 4]</t>
         </is>
       </c>
       <c r="AD40" t="inlineStr">
@@ -7776,7 +7878,7 @@
       </c>
       <c r="AK40" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL40" t="inlineStr">
@@ -7816,6 +7918,7 @@
           <t>An accidental pattern of cell death (morphology) demarcated by cell swelling from failure of plasma-membrane ionic pumps, leading to necrosis with karyolysis.</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -7836,6 +7939,8 @@
           <t>7856735</t>
         </is>
       </c>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr">
         <is>
           <t>Na+/K+-ATPase</t>
@@ -7896,6 +8001,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y41" t="inlineStr"/>
       <c r="Z41" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -7953,7 +8059,7 @@
       </c>
       <c r="AK41" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL41" t="inlineStr">
@@ -8018,6 +8124,7 @@
           <t>29255269</t>
         </is>
       </c>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr">
         <is>
           <t>Oxidative stress-driven, KEAP1/NRF2-dependent</t>
@@ -8083,6 +8190,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y42" t="inlineStr"/>
       <c r="Z42" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -8133,9 +8241,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ42" t="inlineStr"/>
       <c r="AK42" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL42" t="inlineStr">
@@ -8175,6 +8284,7 @@
           <t>An integrated inflammatory cell-death process engaging pyroptosis, apoptosis and necroptosis through the RIPK1/RIPK3-FADD-caspase-8 complex, orchestrated by ZBP1 and TAK1.</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -8195,6 +8305,8 @@
           <t>31850239</t>
         </is>
       </c>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr">
         <is>
           <t>ZBP1, TAK1, RIPK1, RIPK3, FADD, caspase-8, NLRP3</t>
@@ -8255,6 +8367,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y43" t="inlineStr"/>
       <c r="Z43" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -8305,9 +8418,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ43" t="inlineStr"/>
       <c r="AK43" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL43" t="inlineStr">
@@ -8442,6 +8556,7 @@
           <t>DEFINED_RODRIGUES</t>
         </is>
       </c>
+      <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -8492,9 +8607,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ44" t="inlineStr"/>
       <c r="AK44" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL44" t="inlineStr">
@@ -8691,7 +8807,7 @@
       </c>
       <c r="AK45" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL45" t="inlineStr">
@@ -8731,6 +8847,7 @@
           <t>A form of cell death caused by phagocytosis of viable cells, triggered by exposure of 'eat-me' signals or loss of 'don't-eat-me' signals.</t>
         </is>
       </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -8751,6 +8868,8 @@
           <t>22682109</t>
         </is>
       </c>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr">
         <is>
           <t>eat-me signals (PS); CD47</t>
@@ -8811,6 +8930,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y46" t="inlineStr"/>
       <c r="Z46" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -8861,9 +8981,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ46" t="inlineStr"/>
       <c r="AK46" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL46" t="inlineStr">
@@ -8928,6 +9049,9 @@
           <t>14287218</t>
         </is>
       </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>member-dependent</t>
@@ -9015,7 +9139,7 @@
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>LOCKED-VERBATIM</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
@@ -9038,9 +9162,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ47" t="inlineStr"/>
       <c r="AK47" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL47" t="inlineStr">
@@ -9080,6 +9205,7 @@
           <t>A necrosis-like inflammatory cell death of macrophages, executed in a caspase-1-independent manner via ASC and cathepsin B, with release of HMGB1.</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -9100,6 +9226,8 @@
           <t>18005730</t>
         </is>
       </c>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr">
         <is>
           <t>NLRP3, ASC, cathepsin B, HMGB1</t>
@@ -9160,6 +9288,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y48" t="inlineStr"/>
       <c r="Z48" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -9217,7 +9346,7 @@
       </c>
       <c r="AK48" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL48" t="inlineStr">
@@ -9282,6 +9411,7 @@
           <t>26375003;29362479</t>
         </is>
       </c>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>Caspase-1/gasdermin-mediated lysis</t>
@@ -9409,7 +9539,7 @@
       </c>
       <c r="AK49" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL49" t="inlineStr">
@@ -9449,6 +9579,7 @@
           <t>An umbrella term for genetically controlled, non-apoptotic necrotic cell death.</t>
         </is>
       </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -9469,6 +9600,8 @@
           <t>24452471</t>
         </is>
       </c>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr">
         <is>
           <t>RIPK1, RIPK3, MLKL</t>
@@ -9529,6 +9662,7 @@
           <t>DRAFT_CANDIDATE</t>
         </is>
       </c>
+      <c r="Y50" t="inlineStr"/>
       <c r="Z50" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -9586,7 +9720,7 @@
       </c>
       <c r="AK50" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL50" t="inlineStr">
@@ -9626,6 +9760,7 @@
           <t>No single definition - Elicit-derived composite of senescence + autophagy in the cancer context.</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>COMPOSITE</t>
@@ -9646,6 +9781,9 @@
           <t>29362479;36864290</t>
         </is>
       </c>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>not applicable</t>
@@ -9701,6 +9839,7 @@
           <t>COMPOSITE</t>
         </is>
       </c>
+      <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="inlineStr">
         <is>
           <t>COMPOSITE</t>
@@ -9751,9 +9890,10 @@
           <t>associated_with</t>
         </is>
       </c>
+      <c r="AJ51" t="inlineStr"/>
       <c r="AK51" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL51" t="inlineStr">
@@ -9793,6 +9933,7 @@
           <t>A programmed cell death of erythrocytes in which complement activation initiates (mini)NLRP3-caspase-8 complexes culminating in hemolysis.</t>
         </is>
       </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -9813,6 +9954,8 @@
           <t>40252640</t>
         </is>
       </c>
+      <c r="K52" t="inlineStr"/>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>complement; NLRP3; caspase-8</t>
@@ -9873,6 +10016,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -9923,9 +10067,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ52" t="inlineStr"/>
       <c r="AK52" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL52" t="inlineStr">
@@ -9957,7 +10102,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -9965,6 +10110,7 @@
           <t>An endosome-dependent cell-death modality executed through VPS34/PIK3C3 inhibition (oxidation of Cys54/Cys61) and endosomal-identity loss.</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -9977,7 +10123,7 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Tang et al. 2025</t>
+          <t>Swamynathan et al. 2024</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -9985,6 +10131,8 @@
           <t>39446948;39638924</t>
         </is>
       </c>
+      <c r="K53" t="inlineStr"/>
+      <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr">
         <is>
           <t>endosomal machinery</t>
@@ -10045,6 +10193,7 @@
           <t>DRAFT_SOLID</t>
         </is>
       </c>
+      <c r="Y53" t="inlineStr"/>
       <c r="Z53" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -10062,7 +10211,7 @@
       </c>
       <c r="AC53" t="inlineStr">
         <is>
-          <t>Candidate modality (G1+G2 passed; G2 by VPS34 CRISPR-KO + WT-rescue + Cys54/61 non-rescue, PMC11975464); G5 replication pending; human + mouse.</t>
+          <t>Candidate modality (BG1+BG2 passed; BG2 by VPS34 CRISPR-KO + WT-rescue + Cys54/61 non-rescue, PMC11975464); BG5 replication pending; human + mouse.</t>
         </is>
       </c>
       <c r="AD53" t="inlineStr">
@@ -10095,9 +10244,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ53" t="inlineStr"/>
       <c r="AK53" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL53" t="inlineStr">
@@ -10107,7 +10257,7 @@
       </c>
       <c r="AM53" t="inlineStr">
         <is>
-          <t>39638924</t>
+          <t>39446948</t>
         </is>
       </c>
     </row>
@@ -10137,6 +10287,7 @@
           <t>A morphological, taxon-specific pattern of cell death demarcated by conspicuous cytoplasmic vacuolization; in the founding Dictyostelium discoideum (protist) study, autophagy-gene (atg1) disruption reveals a hidden non-vacuolar death pathway, indicating vacuolization is a phenotype rather than the execution mechanism.</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>FOUNDING_DRAFT</t>
@@ -10162,6 +10313,7 @@
           <t>24344187;35390283</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
           <t>atg1</t>
@@ -10222,6 +10374,7 @@
           <t>DRAFT_CANDIDATE</t>
         </is>
       </c>
+      <c r="Y54" t="inlineStr"/>
       <c r="Z54" t="inlineStr">
         <is>
           <t>NOT_IN_NCCD_2018</t>
@@ -10272,9 +10425,10 @@
           <t>root</t>
         </is>
       </c>
+      <c r="AJ54" t="inlineStr"/>
       <c r="AK54" t="inlineStr">
         <is>
-          <t>TRUE; Enrique Medina-Acosta; 2026-09-05</t>
+          <t>TRUE; EM-A (primary) 2026-09-05; HACN (secondary) 2026-09-10; VdSL (secondary) 2026-09-20</t>
         </is>
       </c>
       <c r="AL54" t="inlineStr">
@@ -10289,6 +10443,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>